<commit_message>
dynacmic threshold on rack
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/testbench.xlsx
+++ b/testbench.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BME\lab\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B63E9FE5-CBFB-4BA0-B0DF-0E5D0DEBED20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{671D5B84-A7E5-4647-82BD-F999B2CCF8B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{4B99215D-7811-4DF3-8EAA-804F7E50BB31}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4B99215D-7811-4DF3-8EAA-804F7E50BB31}"/>
   </bookViews>
   <sheets>
     <sheet name="electro" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="55">
   <si>
     <t>LED driver</t>
   </si>
@@ -150,18 +150,12 @@
     <t>CE</t>
   </si>
   <si>
-    <t>LED driver 1</t>
-  </si>
-  <si>
     <t>D3 (PWM)</t>
   </si>
   <si>
     <t>D5 (PWM)</t>
   </si>
   <si>
-    <t>LED driver 2</t>
-  </si>
-  <si>
     <t>CN5711</t>
   </si>
   <si>
@@ -171,9 +165,6 @@
     <t>Név</t>
   </si>
   <si>
-    <t xml:space="preserve">Dióda </t>
-  </si>
-  <si>
     <t>Tiszta nappali fény</t>
   </si>
   <si>
@@ -193,6 +184,24 @@
   </si>
   <si>
     <t>hátulról világító forgalom (?)</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>LED 2</t>
+  </si>
+  <si>
+    <t>LED 1</t>
+  </si>
+  <si>
+    <t>Diódák</t>
+  </si>
+  <si>
+    <t>VCC</t>
+  </si>
+  <si>
+    <t>V5V</t>
   </si>
 </sst>
 </file>
@@ -222,7 +231,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -259,8 +268,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -345,11 +366,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -358,12 +405,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -375,6 +416,26 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -710,262 +771,339 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB089A39-549F-4222-A1B8-B78CE7D21149}">
-  <dimension ref="A4:N26"/>
+  <dimension ref="C4:AD30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.88671875" customWidth="1"/>
-    <col min="3" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="3.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G4" s="1"/>
-      <c r="H4" s="8" t="s">
+    <row r="4" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="J4" s="1"/>
+      <c r="K4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="9"/>
-      <c r="J4" s="1" t="s">
+      <c r="L4" s="13"/>
+      <c r="M4" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G5" s="1" t="s">
+      <c r="Q4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="R4" s="14"/>
+      <c r="S4" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="H5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" s="14"/>
+      <c r="J5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="10"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="8"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G6" s="1"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="1" t="s">
+    <row r="6" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="14"/>
+      <c r="E6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C7" s="5" t="s">
+    <row r="7" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="15"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K7" s="8"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="J8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="8"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="J9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K9" s="8"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="J10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K10" s="8"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P10" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q10" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="R10" s="14"/>
+      <c r="S10" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C11" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="14"/>
+      <c r="E11" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K11" s="8"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="17"/>
+      <c r="Q11" s="19"/>
+      <c r="R11" s="15"/>
+      <c r="S11" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="15"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K12" s="8"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="J13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K13" s="8"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q13" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="R13" s="14"/>
+      <c r="S13" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="J14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K14" s="8"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="19"/>
+      <c r="R14" s="15"/>
+      <c r="S14" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="J15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K15" s="8"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="J16" s="1"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="1"/>
+    </row>
+    <row r="17" spans="8:30" x14ac:dyDescent="0.3">
+      <c r="H17" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I17" s="15"/>
+      <c r="J17" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="K17" s="8"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="1"/>
+    </row>
+    <row r="18" spans="8:30" x14ac:dyDescent="0.3">
+      <c r="J18" s="1"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="1"/>
+    </row>
+    <row r="26" spans="8:30" x14ac:dyDescent="0.3">
+      <c r="AA26" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB26" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AD26" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="8:30" x14ac:dyDescent="0.3">
+      <c r="AA27" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD27" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="8:30" x14ac:dyDescent="0.3">
+      <c r="AA28" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB28" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AC28" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD28" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="8:30" x14ac:dyDescent="0.3">
+      <c r="AA29" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="AB29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="AC29" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD29" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="8:30" x14ac:dyDescent="0.3">
+      <c r="AA30" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB30" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="10"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" s="10"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="10"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" s="10"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" s="10"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="N11" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C12" s="12"/>
-      <c r="D12" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H12" s="10"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" s="10"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="N13" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H14" s="10"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="15" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G15" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H15" s="10"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="G16" s="1"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="G17" s="1"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="1"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="G18" s="1"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="1"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="1" t="s">
+      <c r="AC30" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD30" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="H4:I18"/>
-    <mergeCell ref="C11:C12"/>
+  <mergeCells count="8">
+    <mergeCell ref="Q10:Q11"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="Q13:Q14"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="P10:P11"/>
+    <mergeCell ref="P13:P14"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="E11:E12"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -987,13 +1125,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1001,13 +1139,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1015,13 +1153,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
         <v>47</v>
       </c>
-      <c r="C4" t="s">
-        <v>50</v>
-      </c>
       <c r="D4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1029,13 +1167,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" t="s">
         <v>48</v>
-      </c>
-      <c r="C5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1043,13 +1181,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1058,6 +1196,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentum" ma:contentTypeID="0x0101002791E5C9BFFA5B4A81D7C4A231B254C2" ma:contentTypeVersion="9" ma:contentTypeDescription="Új dokumentum létrehozása." ma:contentTypeScope="" ma:versionID="05f77945d41b57df2bd29514a2af1f0b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="fde77160-36ee-44b4-844a-718fc8dda880" xmlns:ns4="1ec56c6a-bd3e-4b9c-bbdf-18231c25e385" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5695c1091b184db45d7fd427357a4edf" ns3:_="" ns4:_="">
     <xsd:import namespace="fde77160-36ee-44b4-844a-718fc8dda880"/>
@@ -1252,15 +1399,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1270,6 +1408,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9322816-506E-4289-B7C4-09DB39F46D43}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36346629-4145-4987-B1BA-59BF87F392EF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1284,14 +1430,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9322816-506E-4289-B7C4-09DB39F46D43}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>